<commit_message>
Se actualizan scripts para paquete 2
</commit_message>
<xml_diff>
--- a/tests/automatizacion api/serenity rest/src/test/resources/datadriven/datadriven.xlsx
+++ b/tests/automatizacion api/serenity rest/src/test/resources/datadriven/datadriven.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jherrodr\Downloads\EverestAutomatizacion\demo-servicios-axet-plugin1\tests\automatizacion api\serenity rest\src\test\resources\datadriven\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jherrodr\Downloads\EverestAutomatizacion\demo-servicios-axet-plugin\tests\automatizacion api\serenity rest\src\test\resources\datadriven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B733F901-9DAB-47D7-9020-2F4A6D23AABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA0CF1A-674B-40EF-A3EE-F5257CDC7D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="retiro" sheetId="1" state="hidden" r:id="rId1"/>
@@ -184,7 +184,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2965" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="431">
   <si>
     <t>Caso</t>
   </si>
@@ -1326,15 +1326,9 @@
     <t>55555555-5555-5555-5555-555555555555</t>
   </si>
   <si>
-    <t>2222222222222222</t>
-  </si>
-  <si>
     <t>00000000-0000-0000-0000-000000000504</t>
   </si>
   <si>
-    <t>3333333333333333</t>
-  </si>
-  <si>
     <t>trace-bpop-ok-001</t>
   </si>
   <si>
@@ -1468,6 +1462,21 @@
   </si>
   <si>
     <t>trace-avv-op-invalid-001</t>
+  </si>
+  <si>
+    <t>0000000000000504</t>
+  </si>
+  <si>
+    <t>1234-5678-9012-3456</t>
+  </si>
+  <si>
+    <t>4444444444444444</t>
+  </si>
+  <si>
+    <t>4000000000000504</t>
+  </si>
+  <si>
+    <t>trace-hu203-bpop-502</t>
   </si>
 </sst>
 </file>
@@ -2684,7 +2693,7 @@
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="17" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="L8" s="14" t="s">
         <v>343</v>
@@ -3077,7 +3086,7 @@
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="17" t="s">
-        <v>380</v>
+        <v>428</v>
       </c>
       <c r="L7" s="14" t="s">
         <v>343</v>
@@ -3127,7 +3136,7 @@
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="17" t="s">
-        <v>380</v>
+        <v>428</v>
       </c>
       <c r="L8" s="14" t="s">
         <v>343</v>
@@ -3158,7 +3167,7 @@
         <v>338</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>352</v>
+        <v>378</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>277</v>
@@ -3177,7 +3186,7 @@
       </c>
       <c r="J9" s="14"/>
       <c r="K9" s="17" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="L9" s="14" t="s">
         <v>343</v>
@@ -3621,7 +3630,7 @@
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="17" t="s">
-        <v>382</v>
+        <v>426</v>
       </c>
       <c r="L8" s="14" t="s">
         <v>343</v>
@@ -4378,7 +4387,7 @@
         <v>338</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>277</v>
@@ -4404,8 +4413,8 @@
       <c r="N7" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="O7" s="14" t="s">
-        <v>362</v>
+      <c r="O7" s="14">
+        <v>3000000504</v>
       </c>
       <c r="P7" s="14" t="s">
         <v>363</v>
@@ -4737,7 +4746,7 @@
         <v>338</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>378</v>
+        <v>430</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>277</v>
@@ -4751,8 +4760,8 @@
       <c r="H6" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="14" t="s">
-        <v>353</v>
+      <c r="I6" s="14">
+        <v>99999999</v>
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
@@ -4763,8 +4772,8 @@
       <c r="N6" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="O6" s="14" t="s">
-        <v>362</v>
+      <c r="O6" s="14">
+        <v>4000000502</v>
       </c>
       <c r="P6" s="14" t="s">
         <v>363</v>
@@ -4817,8 +4826,8 @@
       <c r="N7" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="O7" s="14" t="s">
-        <v>362</v>
+      <c r="O7" s="14">
+        <v>3000000504</v>
       </c>
       <c r="P7" s="14" t="s">
         <v>363</v>
@@ -12120,7 +12129,7 @@
         <v>338</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>326</v>
@@ -12129,7 +12138,7 @@
         <v>326</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>18</v>
@@ -12138,7 +12147,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K2" s="17" t="s">
         <v>343</v>
@@ -12164,7 +12173,7 @@
         <v>338</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>326</v>
@@ -12173,7 +12182,7 @@
         <v>326</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>18</v>
@@ -12182,7 +12191,7 @@
         <v>19</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="K3" s="17" t="s">
         <v>343</v>
@@ -12194,7 +12203,7 @@
         <v>265</v>
       </c>
       <c r="N3" s="14" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12208,7 +12217,7 @@
         <v>338</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>326</v>
@@ -12217,7 +12226,7 @@
         <v>326</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H4" s="14" t="s">
         <v>18</v>
@@ -12226,7 +12235,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="K4" s="17" t="s">
         <v>343</v>
@@ -12238,7 +12247,7 @@
         <v>35</v>
       </c>
       <c r="N4" s="14" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12252,7 +12261,7 @@
         <v>338</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>326</v>
@@ -12270,7 +12279,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K5" s="17" t="s">
         <v>343</v>
@@ -12371,7 +12380,7 @@
         <v>338</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>277</v>
@@ -12380,7 +12389,7 @@
         <v>277</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>18</v>
@@ -12389,7 +12398,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>343</v>
@@ -12415,7 +12424,7 @@
         <v>338</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>277</v>
@@ -12424,7 +12433,7 @@
         <v>277</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>18</v>
@@ -12432,7 +12441,9 @@
       <c r="I3" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="14"/>
+      <c r="J3" s="14" t="s">
+        <v>427</v>
+      </c>
       <c r="K3" s="14" t="s">
         <v>343</v>
       </c>
@@ -12443,7 +12454,7 @@
         <v>321</v>
       </c>
       <c r="N3" s="14" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12457,7 +12468,7 @@
         <v>338</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>277</v>
@@ -12466,7 +12477,7 @@
         <v>277</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H4" s="14" t="s">
         <v>18</v>
@@ -12474,8 +12485,8 @@
       <c r="I4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="14" t="s">
-        <v>385</v>
+      <c r="J4" s="17" t="s">
+        <v>388</v>
       </c>
       <c r="K4" s="14" t="s">
         <v>343</v>
@@ -12487,7 +12498,7 @@
         <v>35</v>
       </c>
       <c r="N4" s="14" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12501,7 +12512,7 @@
         <v>338</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>277</v>
@@ -12510,7 +12521,7 @@
         <v>277</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H5" s="14" t="s">
         <v>18</v>
@@ -12531,7 +12542,7 @@
         <v>298</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12545,7 +12556,7 @@
         <v>338</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>277</v>
@@ -12554,7 +12565,7 @@
         <v>277</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>18</v>
@@ -12575,7 +12586,7 @@
         <v>34</v>
       </c>
       <c r="N6" s="14" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12589,7 +12600,7 @@
         <v>338</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>277</v>
@@ -12598,7 +12609,7 @@
         <v>277</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>18</v>
@@ -12606,8 +12617,8 @@
       <c r="I7" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="14" t="s">
-        <v>385</v>
+      <c r="J7" s="17" t="s">
+        <v>388</v>
       </c>
       <c r="K7" s="14" t="s">
         <v>343</v>
@@ -12619,7 +12630,7 @@
         <v>35</v>
       </c>
       <c r="N7" s="14" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12633,7 +12644,7 @@
         <v>338</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>277</v>
@@ -12651,7 +12662,7 @@
         <v>19</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K8" s="14" t="s">
         <v>343</v>
@@ -12727,7 +12738,7 @@
         <v>332</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K1" s="12" t="s">
         <v>14</v>
@@ -12750,7 +12761,7 @@
         <v>338</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>314</v>
@@ -12759,16 +12770,16 @@
         <v>314</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I2" s="14" t="s">
         <v>343</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K2" s="17">
         <v>200</v>
@@ -12791,7 +12802,7 @@
         <v>338</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>314</v>
@@ -12800,7 +12811,7 @@
         <v>314</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>304</v>
@@ -12809,7 +12820,7 @@
         <v>343</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K3" s="17">
         <v>422</v>
@@ -12818,7 +12829,7 @@
         <v>298</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12832,7 +12843,7 @@
         <v>338</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>314</v>
@@ -12841,16 +12852,16 @@
         <v>314</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="I4" s="14" t="s">
         <v>343</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K4" s="17">
         <v>200</v>
@@ -12859,7 +12870,7 @@
         <v>29</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12873,7 +12884,7 @@
         <v>338</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>314</v>
@@ -12882,16 +12893,16 @@
         <v>314</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>384</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>385</v>
+        <v>382</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>348</v>
       </c>
       <c r="I5" s="14" t="s">
         <v>343</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K5" s="17">
         <v>502</v>
@@ -12900,7 +12911,7 @@
         <v>34</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12914,7 +12925,7 @@
         <v>338</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>314</v>
@@ -12923,16 +12934,16 @@
         <v>314</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>384</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>385</v>
+        <v>382</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>348</v>
       </c>
       <c r="I6" s="14" t="s">
         <v>343</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K6" s="17">
         <v>502</v>
@@ -12941,7 +12952,7 @@
         <v>34</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12955,7 +12966,7 @@
         <v>338</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>314</v>
@@ -12964,16 +12975,16 @@
         <v>314</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>384</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>385</v>
+        <v>382</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>388</v>
       </c>
       <c r="I7" s="14" t="s">
         <v>343</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K7" s="17">
         <v>504</v>
@@ -12982,7 +12993,7 @@
         <v>35</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -12996,7 +13007,7 @@
         <v>338</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>314</v>
@@ -13005,16 +13016,16 @@
         <v>314</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>384</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>385</v>
+        <v>382</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>388</v>
       </c>
       <c r="I8" s="14" t="s">
         <v>343</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K8" s="17">
         <v>504</v>
@@ -13023,7 +13034,7 @@
         <v>35</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -13110,7 +13121,7 @@
         <v>338</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>23</v>
@@ -13119,7 +13130,7 @@
         <v>23</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>18</v>
@@ -13128,7 +13139,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K2" s="14">
         <v>200</v>
@@ -13151,7 +13162,7 @@
         <v>338</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>23</v>
@@ -13160,16 +13171,16 @@
         <v>23</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>18</v>
       </c>
       <c r="I3" s="14" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K3" s="14">
         <v>422</v>
@@ -13192,7 +13203,7 @@
         <v>338</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>23</v>
@@ -13201,16 +13212,16 @@
         <v>23</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H4" s="14" t="s">
         <v>18</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K4" s="14">
         <v>502</v>
@@ -13219,7 +13230,7 @@
         <v>34</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -13233,7 +13244,7 @@
         <v>338</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>23</v>
@@ -13242,16 +13253,16 @@
         <v>23</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="H5" s="14" t="s">
         <v>18</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K5" s="14">
         <v>504</v>
@@ -13260,7 +13271,7 @@
         <v>35</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -13274,7 +13285,7 @@
         <v>338</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>23</v>
@@ -13292,7 +13303,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K6" s="14">
         <v>400</v>

</xml_diff>